<commit_message>
Corrida | GSF-TD | 2026-07-14 09:01:53.128406
</commit_message>
<xml_diff>
--- a/indicadores/GSF-TD_out.xlsx
+++ b/indicadores/GSF-TD_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">13/07/2026</t>
+    <t xml:space="preserve">14/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">vcorvalan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>